<commit_message>
Actualización del archivo "analisis_OC.xlsx" para reflejar cambios en el análisis de datos. Se han realizado modificaciones significativas en el contenido del archivo.
</commit_message>
<xml_diff>
--- a/analisis_OC.xlsx
+++ b/analisis_OC.xlsx
@@ -17,17 +17,44 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={0c2c9d05-a49b-4935-a225-17c66f09b0d7}</author>
-    <author>tc={2d4f0503-db14-4fa0-aed9-4eed0b8060d3}</author>
-    <author>tc={4240f779-182c-41a1-b086-924dbb0002c4}</author>
-    <author>tc={4ee4de7c-9ee8-485b-b1f6-e46c7ec6b5e5}</author>
-    <author>tc={52912bc3-eefb-4b27-ace6-7a42c55f9736}</author>
-    <author>tc={75253bad-0f41-40ff-a930-8872ee6f1d16}</author>
-    <author>tc={ac850828-3741-4830-8e95-3fd909fae070}</author>
-    <author>tc={bca4589b-31b6-4632-875d-445911a70f78}</author>
+    <author>tc={0774e333-b72f-4495-8fad-e55243485ff2}</author>
+    <author>tc={1ddaf5b2-0bd8-4ba0-96bf-ea112996fee1}</author>
+    <author>tc={23b712ab-60b5-4c7a-8e10-ec20f5b80aa0}</author>
+    <author>tc={3920ed91-4b87-44b2-b179-e18db364969d}</author>
+    <author>tc={71924a42-280b-47e8-badc-42cf8041cd83}</author>
+    <author>tc={85af4a8e-49cf-4434-b95c-35396a30103f}</author>
+    <author>tc={95f0565e-9b91-464c-90e6-dcb20b5cd991}</author>
+    <author>tc={e580cd2a-44c1-46da-852d-b48bbb81e74e}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{0c2c9d05-a49b-4935-a225-17c66f09b0d7}" ref="B1">
+    <comment authorId="0" xr:uid="{0774e333-b72f-4495-8fad-e55243485ff2}" ref="E1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	El tiempo en días a la semana que el proveedor viene a entregar mercancia
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{1ddaf5b2-0bd8-4ba0-96bf-ea112996fee1}" ref="E1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	El tiempo en la semana que el proveedor viene a entregar mercancia
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{23b712ab-60b5-4c7a-8e10-ec20f5b80aa0}" ref="G1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Cantidad e ventas por semanas, necesario para el promedio de venta. (SEM1-SEM5)
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{3920ed91-4b87-44b2-b179-e18db364969d}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -36,7 +63,25 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{2d4f0503-db14-4fa0-aed9-4eed0b8060d3}" ref="C1">
+    <comment authorId="4" xr:uid="{71924a42-280b-47e8-badc-42cf8041cd83}" ref="A1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Código que uses para identificar el producto.
+</t>
+      </text>
+    </comment>
+    <comment authorId="5" xr:uid="{85af4a8e-49cf-4434-b95c-35396a30103f}" ref="D1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	El inventario neto de tu almacén.
+</t>
+      </text>
+    </comment>
+    <comment authorId="6" xr:uid="{95f0565e-9b91-464c-90e6-dcb20b5cd991}" ref="C1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -45,16 +90,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{4240f779-182c-41a1-b086-924dbb0002c4}" ref="A1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Código que uses para identificar el producto.
-</t>
-      </text>
-    </comment>
-    <comment authorId="3" xr:uid="{4ee4de7c-9ee8-485b-b1f6-e46c7ec6b5e5}" ref="F1">
+    <comment authorId="7" xr:uid="{e580cd2a-44c1-46da-852d-b48bbb81e74e}" ref="F1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,48 +99,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="4" xr:uid="{52912bc3-eefb-4b27-ace6-7a42c55f9736}" ref="D1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	El inventario neto de tu almacén.
-</t>
-      </text>
-    </comment>
-    <comment authorId="5" xr:uid="{75253bad-0f41-40ff-a930-8872ee6f1d16}" ref="G1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Cantidad e ventas por semanas, necesario para el promedio de venta. (SEM1-SEM5)
-</t>
-      </text>
-    </comment>
-    <comment authorId="6" xr:uid="{ac850828-3741-4830-8e95-3fd909fae070}" ref="E1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	El tiempo en días a la semana que el proveedor viene a entregar mercancia
-</t>
-      </text>
-    </comment>
-    <comment authorId="7" xr:uid="{bca4589b-31b6-4632-875d-445911a70f78}" ref="E1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	El tiempo en la semana que el proveedor viene a entregar mercancia
-</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>codigo</t>
   </si>
@@ -139,52 +139,7 @@
     <t>SEM5</t>
   </si>
   <si>
-    <t>100837035</t>
-  </si>
-  <si>
-    <t>Pan De Tata Sandwich Paq.575Gr</t>
-  </si>
-  <si>
-    <t>100837043</t>
-  </si>
-  <si>
-    <t>Pan De Tata Para Perro Caliente Paq.8Und</t>
-  </si>
-  <si>
-    <t>100837051</t>
-  </si>
-  <si>
-    <t>Mini Pan De Tata Para Hamburguesa Paq.15Und</t>
-  </si>
-  <si>
-    <t>100837060</t>
-  </si>
-  <si>
-    <t>Pan De Tata Para Hamburgresa Paq.6Und</t>
-  </si>
-  <si>
-    <t>100837078</t>
-  </si>
-  <si>
-    <t>Pan De Tata Tipo Deli Paq.4und</t>
-  </si>
-  <si>
-    <t>100905228</t>
-  </si>
-  <si>
-    <t>Pan De Tata Molido Paquete 300Gr</t>
-  </si>
-  <si>
-    <t>100905663</t>
-  </si>
-  <si>
-    <t>Porquecitos De Tata Doraditos Paq. 12 Und  540Gr</t>
-  </si>
-  <si>
-    <t>100904772</t>
-  </si>
-  <si>
-    <t>Ponque De Tata Paquete 450Gr</t>
+    <t>informacion sobre los productos</t>
   </si>
   <si>
     <t>Columnas</t>
@@ -311,7 +266,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Bryant Facenda" id="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" providerId="google-sheets"/>
+  <x18tc:person displayName="Bryant Facenda" id="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -322,97 +277,59 @@
   </cacheSource>
   <cacheFields>
     <cacheField name="codigo" numFmtId="0">
-      <sharedItems>
-        <s v="100837035"/>
-        <s v="100837043"/>
-        <s v="100837051"/>
-        <s v="100837060"/>
-        <s v="100837078"/>
-        <s v="100905228"/>
-        <s v="100905663"/>
-        <s v="100904772"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="descripcion" numFmtId="0">
-      <sharedItems>
-        <s v="Pan De Tata Sandwich Paq.575Gr"/>
-        <s v="Pan De Tata Para Perro Caliente Paq.8Und"/>
-        <s v="Mini Pan De Tata Para Hamburguesa Paq.15Und"/>
-        <s v="Pan De Tata Para Hamburgresa Paq.6Und"/>
-        <s v="Pan De Tata Tipo Deli Paq.4und"/>
-        <s v="Pan De Tata Molido Paquete 300Gr"/>
-        <s v="Porquecitos De Tata Doraditos Paq. 12 Und  540Gr"/>
-        <s v="Ponque De Tata Paquete 450Gr"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="empaque" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="1.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="cantidad_en_mano" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="9.0"/>
-        <n v="4.0"/>
-        <n v="3.0"/>
-        <n v="1.0"/>
-        <n v="5.0"/>
-        <n v="2.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="tiempo_reposicion" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="1.0"/>
+      <sharedItems containsBlank="1">
+        <s v="informacion sobre los productos"/>
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="stock_seguridad" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="10.0"/>
-        <n v="7.0"/>
-        <n v="3.0"/>
-        <n v="2.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="SEM1" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="3.0"/>
-        <n v="0.0"/>
-        <n v="2.0"/>
-        <n v="1.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="SEM2" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="10.0"/>
-        <n v="7.0"/>
-        <n v="1.0"/>
-        <n v="5.0"/>
-        <n v="3.0"/>
-        <n v="0.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="SEM3" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="12.0"/>
-        <n v="7.0"/>
-        <n v="3.0"/>
-        <n v="14.0"/>
-        <n v="2.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="SEM4" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="4.0"/>
-        <n v="6.0"/>
-        <n v="2.0"/>
-        <n v="11.0"/>
-        <n v="0.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
     <cacheField name="SEM5" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
-        <n v="1.0"/>
-        <n v="0.0"/>
+      <sharedItems containsString="0" containsBlank="1">
+        <m/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -426,26 +343,12 @@
     <pivotField name="codigo" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="descripcion" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -458,73 +361,49 @@
     <pivotField name="cantidad_en_mano" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="tiempo_reposicion" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="stock_seguridad" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="SEM1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="SEM2" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="SEM3" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="SEM4" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField name="SEM5" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
       <items>
         <item x="0"/>
-        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -728,28 +607,28 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-07-22T14:26:00.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{0c2c9d05-a49b-4935-a225-17c66f09b0d7}" done="0">
+  <x18tc:threadedComment ref="B1" dT="2026-07-22T14:26:00.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{3920ed91-4b87-44b2-b179-e18db364969d}" done="0">
     <x18tc:text xml:space="preserve">Descripcion del producto</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E1" dT="2026-07-22T14:28:02.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{ac850828-3741-4830-8e95-3fd909fae070}" done="1">
+  <x18tc:threadedComment ref="E1" dT="2026-07-22T14:28:02.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{0774e333-b72f-4495-8fad-e55243485ff2}" done="1">
     <x18tc:text xml:space="preserve">El tiempo en días a la semana que el proveedor viene a entregar mercancia</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A1" dT="2026-07-22T14:25:31.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{4240f779-182c-41a1-b086-924dbb0002c4}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-07-22T14:25:31.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{71924a42-280b-47e8-badc-42cf8041cd83}" done="0">
     <x18tc:text xml:space="preserve">Código que uses para identificar el producto.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E1" dT="2026-07-22T14:31:32.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{bca4589b-31b6-4632-875d-445911a70f78}" done="0">
+  <x18tc:threadedComment ref="E1" dT="2026-07-22T14:31:32.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{1ddaf5b2-0bd8-4ba0-96bf-ea112996fee1}" done="0">
     <x18tc:text xml:space="preserve">El tiempo en la semana que el proveedor viene a entregar mercancia</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="D1" dT="2026-07-22T14:27:04.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{52912bc3-eefb-4b27-ace6-7a42c55f9736}" done="0">
+  <x18tc:threadedComment ref="D1" dT="2026-07-22T14:27:04.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{85af4a8e-49cf-4434-b95c-35396a30103f}" done="0">
     <x18tc:text xml:space="preserve">El inventario neto de tu almacén.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="G1" dT="2026-07-22T14:32:37.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{75253bad-0f41-40ff-a930-8872ee6f1d16}" done="0">
+  <x18tc:threadedComment ref="G1" dT="2026-07-22T14:32:37.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{23b712ab-60b5-4c7a-8e10-ec20f5b80aa0}" done="0">
     <x18tc:text xml:space="preserve">Cantidad e ventas por semanas, necesario para el promedio de venta. (SEM1-SEM5)</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="F1" dT="2026-07-22T14:30:20.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{4ee4de7c-9ee8-485b-b1f6-e46c7ec6b5e5}" done="0">
+  <x18tc:threadedComment ref="F1" dT="2026-07-22T14:30:20.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{e580cd2a-44c1-46da-852d-b48bbb81e74e}" done="0">
     <x18tc:text xml:space="preserve">Cantidad colchon ante cualquier eventualidad con el proveedor. (puede ser la cantidad mínima permitida de tu inventario )</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="C1" dT="2026-07-22T14:26:41.00" personId="{d1b7703b-91c1-4366-a7ed-a37fb700ef5b}" id="{2d4f0503-db14-4fa0-aed9-4eed0b8060d3}" done="0">
+  <x18tc:threadedComment ref="C1" dT="2026-07-22T14:26:41.00" personId="{9e0ac0c1-578c-4303-9cd3-c0ec2eed338f}" id="{95f0565e-9b91-464c-90e6-dcb20b5cd991}" done="0">
     <x18tc:text xml:space="preserve">El tamaño del empaque del producto, útil para calcular el pedido en empaque para el proveedor.</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -806,284 +685,110 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D2" s="4">
-        <v>9.0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F2" s="4">
-        <v>10.0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="H2" s="4">
-        <v>10.0</v>
-      </c>
-      <c r="I2" s="4">
-        <v>12.0</v>
-      </c>
-      <c r="J2" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="K2" s="4">
-        <v>1.0</v>
-      </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D3" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E3" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F3" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="G3" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="H3" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="I3" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="J3" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="K3" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D4" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F4" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="H4" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="I4" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="J4" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F5" s="4">
-        <v>10.0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="H5" s="4">
-        <v>10.0</v>
-      </c>
-      <c r="I5" s="4">
-        <v>14.0</v>
-      </c>
-      <c r="J5" s="4">
-        <v>11.0</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F6" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="H6" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="I6" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="J6" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K6" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D7" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="E7" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F7" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="H7" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="I7" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="J7" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="K7" s="4">
-        <v>1.0</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D8" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="E8" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F8" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="H8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="I8" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K8" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="D9" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="E9" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F9" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="H9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="I9" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="J9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K9" s="4">
-        <v>0.0</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
     </row>
     <row r="10">
       <c r="B10" s="7"/>

</xml_diff>